<commit_message>
fix(samples): the sample workbook is input only
Expected_Output is not something a client produces. In the handoff template
that tab describes the allocation sheet the engine *emits* — export-allocation.ts
already keeps its column order — so shipping a sample that contained one taught
the wrong thing about the input format.

The tab is gone. The workbook now carries Fund_Setup, LP_Register,
Call_Components, Management_Fee and Transfers, and nothing else; a test asserts
that list, so one cannot creep back in.

The figures it held are now assertions in the test, still taken from the
delivered spec engine rather than from this one. A failure names the investor
and the column:

  AssertionError: LP01 · Total_Call: expected 2943299.99 to be close to
  2943399.99, received difference is 100

Verified by perturbing one figure by 100 dollars.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/meridian-growth-partners-iii-call-4.xlsx
+++ b/samples/meridian-growth-partners-iii-call-4.xlsx
@@ -9,7 +9,6 @@
     <sheet name="Call_Components" sheetId="4" r:id="rId4"/>
     <sheet name="Management_Fee" sheetId="5" r:id="rId5"/>
     <sheet name="Transfers" sheetId="6" r:id="rId6"/>
-    <sheet name="Expected_Output" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -403,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,22 +456,32 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v xml:space="preserve">  Expected_Output   Regression fixture. The engine checks its result against it.</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
+        <v>This tab, and any tab not listed above, is ignored.</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>This tab, and any tab not listed above, is ignored.</v>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>There is no expected-output tab: the allocation sheet is what the app</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>produces from these inputs, not something you fill in.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1641,687 +1650,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Expected Output — golden test case</v>
-      </c>
-      <c r="B1" t="str">
-        <v/>
-      </c>
-      <c r="C1" t="str">
-        <v/>
-      </c>
-      <c r="D1" t="str">
-        <v/>
-      </c>
-      <c r="E1" t="str">
-        <v/>
-      </c>
-      <c r="F1" t="str">
-        <v/>
-      </c>
-      <c r="G1" t="str">
-        <v/>
-      </c>
-      <c r="H1" t="str">
-        <v/>
-      </c>
-      <c r="I1" t="str">
-        <v/>
-      </c>
-      <c r="J1" t="str">
-        <v/>
-      </c>
-      <c r="K1" t="str">
-        <v/>
-      </c>
-      <c r="L1" t="str">
-        <v/>
-      </c>
-      <c r="M1" t="str">
-        <v/>
-      </c>
-      <c r="N1" t="str">
-        <v/>
-      </c>
-      <c r="O1" t="str">
-        <v/>
-      </c>
-      <c r="P1" t="str">
-        <v/>
-      </c>
-      <c r="Q1" t="str">
-        <v/>
-      </c>
-      <c r="R1" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Figures produced by the delivered spec engine. The app checks its own result against them.</v>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v/>
-      </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v/>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>LP_ID</v>
-      </c>
-      <c r="B3" t="str">
-        <v>LP_Name</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Commitment</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Opening_UCC</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Opening_Paid_In</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Project_Helios</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Project_Orion</v>
-      </c>
-      <c r="H3" t="str">
-        <v>Bridge_Facility_Repayment</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Fund_Operating_Expenses</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Formation_Cost_True_Up</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Fee_Rate</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Fee_Gross</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Fee_Offset</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Fee_Net</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Total_Call</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Reduces_Unfunded_Amt</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Closing_UCC</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Closing_Paid_In</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>LP01</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Northbridge Retirement System</v>
-      </c>
-      <c r="C4">
-        <v>25000000</v>
-      </c>
-      <c r="D4">
-        <v>16250000</v>
-      </c>
-      <c r="E4">
-        <v>8750000</v>
-      </c>
-      <c r="F4">
-        <v>1614583.33</v>
-      </c>
-      <c r="G4">
-        <v>885416.67</v>
-      </c>
-      <c r="H4">
-        <v>325520.83</v>
-      </c>
-      <c r="I4">
-        <v>74218.75</v>
-      </c>
-      <c r="J4">
-        <v>31250</v>
-      </c>
-      <c r="K4">
-        <v>0.0175</v>
-      </c>
-      <c r="L4">
-        <v>33687.5</v>
-      </c>
-      <c r="M4">
-        <v>21377.09</v>
-      </c>
-      <c r="N4">
-        <v>12310.41</v>
-      </c>
-      <c r="O4">
-        <v>2943299.99</v>
-      </c>
-      <c r="P4">
-        <v>2912049.99</v>
-      </c>
-      <c r="Q4">
-        <v>13337950.01</v>
-      </c>
-      <c r="R4">
-        <v>11693299.99</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>LP02</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Kestrel University Endowment</v>
-      </c>
-      <c r="C5">
-        <v>12000000</v>
-      </c>
-      <c r="D5">
-        <v>7800000</v>
-      </c>
-      <c r="E5">
-        <v>4200000</v>
-      </c>
-      <c r="F5">
-        <v>775000</v>
-      </c>
-      <c r="G5">
-        <v>425000</v>
-      </c>
-      <c r="H5">
-        <v>156250</v>
-      </c>
-      <c r="I5">
-        <v>35625</v>
-      </c>
-      <c r="J5">
-        <v>15000</v>
-      </c>
-      <c r="K5">
-        <v>0.0175</v>
-      </c>
-      <c r="L5">
-        <v>16170</v>
-      </c>
-      <c r="M5">
-        <v>10261.01</v>
-      </c>
-      <c r="N5">
-        <v>5908.99</v>
-      </c>
-      <c r="O5">
-        <v>1412783.99</v>
-      </c>
-      <c r="P5">
-        <v>1397783.99</v>
-      </c>
-      <c r="Q5">
-        <v>6402216.01</v>
-      </c>
-      <c r="R5">
-        <v>5612783.99</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>LP03</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Tanaka Family Holdings KK</v>
-      </c>
-      <c r="C6">
-        <v>6000000</v>
-      </c>
-      <c r="D6">
-        <v>3900000</v>
-      </c>
-      <c r="E6">
-        <v>2100000</v>
-      </c>
-      <c r="F6">
-        <v>387500</v>
-      </c>
-      <c r="G6">
-        <v>212500</v>
-      </c>
-      <c r="H6">
-        <v>78125</v>
-      </c>
-      <c r="I6">
-        <v>17812.5</v>
-      </c>
-      <c r="J6">
-        <v>7500</v>
-      </c>
-      <c r="K6">
-        <v>0.015</v>
-      </c>
-      <c r="L6">
-        <v>6930</v>
-      </c>
-      <c r="M6">
-        <v>4397.57</v>
-      </c>
-      <c r="N6">
-        <v>2532.43</v>
-      </c>
-      <c r="O6">
-        <v>705969.93</v>
-      </c>
-      <c r="P6">
-        <v>698469.93</v>
-      </c>
-      <c r="Q6">
-        <v>3201530.07</v>
-      </c>
-      <c r="R6">
-        <v>2805969.93</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>LP04</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Arbor Mutual Assurance</v>
-      </c>
-      <c r="C7">
-        <v>30000000</v>
-      </c>
-      <c r="D7">
-        <v>19500000</v>
-      </c>
-      <c r="E7">
-        <v>10500000</v>
-      </c>
-      <c r="F7">
-        <v>1937500</v>
-      </c>
-      <c r="G7">
-        <v>1062500</v>
-      </c>
-      <c r="H7">
-        <v>390625</v>
-      </c>
-      <c r="I7">
-        <v>89062.49</v>
-      </c>
-      <c r="J7">
-        <v>37500</v>
-      </c>
-      <c r="K7">
-        <v>0.0175</v>
-      </c>
-      <c r="L7">
-        <v>40425</v>
-      </c>
-      <c r="M7">
-        <v>25652.5</v>
-      </c>
-      <c r="N7">
-        <v>14772.5</v>
-      </c>
-      <c r="O7">
-        <v>3531959.99</v>
-      </c>
-      <c r="P7">
-        <v>3494459.99</v>
-      </c>
-      <c r="Q7">
-        <v>16005540.01</v>
-      </c>
-      <c r="R7">
-        <v>14031959.99</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>LP05</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Halvorsen Nominees Limited</v>
-      </c>
-      <c r="C8">
-        <v>9500000</v>
-      </c>
-      <c r="D8">
-        <v>6175000</v>
-      </c>
-      <c r="E8">
-        <v>3325000</v>
-      </c>
-      <c r="F8">
-        <v>613541.67</v>
-      </c>
-      <c r="G8">
-        <v>336458.33</v>
-      </c>
-      <c r="H8">
-        <v>123697.92</v>
-      </c>
-      <c r="I8">
-        <v>28203.13</v>
-      </c>
-      <c r="J8">
-        <v>11875</v>
-      </c>
-      <c r="K8">
-        <v>0.0175</v>
-      </c>
-      <c r="L8">
-        <v>12801.25</v>
-      </c>
-      <c r="M8">
-        <v>8123.29</v>
-      </c>
-      <c r="N8">
-        <v>4677.96</v>
-      </c>
-      <c r="O8">
-        <v>1118454.01</v>
-      </c>
-      <c r="P8">
-        <v>1106579.01</v>
-      </c>
-      <c r="Q8">
-        <v>5068420.99</v>
-      </c>
-      <c r="R8">
-        <v>4443454.01</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>LP06</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Sycamore Foundation</v>
-      </c>
-      <c r="C9">
-        <v>4500000</v>
-      </c>
-      <c r="D9">
-        <v>2925000</v>
-      </c>
-      <c r="E9">
-        <v>1575000</v>
-      </c>
-      <c r="F9">
-        <v>290625</v>
-      </c>
-      <c r="G9">
-        <v>159375</v>
-      </c>
-      <c r="H9">
-        <v>58593.75</v>
-      </c>
-      <c r="I9">
-        <v>13359.38</v>
-      </c>
-      <c r="J9">
-        <v>5625</v>
-      </c>
-      <c r="K9">
-        <v>0.0175</v>
-      </c>
-      <c r="L9">
-        <v>6063.75</v>
-      </c>
-      <c r="M9">
-        <v>3847.87</v>
-      </c>
-      <c r="N9">
-        <v>2215.88</v>
-      </c>
-      <c r="O9">
-        <v>529794.01</v>
-      </c>
-      <c r="P9">
-        <v>524169.01</v>
-      </c>
-      <c r="Q9">
-        <v>2400830.99</v>
-      </c>
-      <c r="R9">
-        <v>2104794.01</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>LP07</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Bridgeline Capital SCSp</v>
-      </c>
-      <c r="C10">
-        <v>8000000</v>
-      </c>
-      <c r="D10">
-        <v>5200000</v>
-      </c>
-      <c r="E10">
-        <v>2800000</v>
-      </c>
-      <c r="F10">
-        <v>516666.67</v>
-      </c>
-      <c r="G10">
-        <v>283333.33</v>
-      </c>
-      <c r="H10">
-        <v>104166.67</v>
-      </c>
-      <c r="I10">
-        <v>23750</v>
-      </c>
-      <c r="J10">
-        <v>10000</v>
-      </c>
-      <c r="K10">
-        <v>0.0175</v>
-      </c>
-      <c r="L10">
-        <v>10780</v>
-      </c>
-      <c r="M10">
-        <v>6840.67</v>
-      </c>
-      <c r="N10">
-        <v>3939.33</v>
-      </c>
-      <c r="O10">
-        <v>941856</v>
-      </c>
-      <c r="P10">
-        <v>931856</v>
-      </c>
-      <c r="Q10">
-        <v>4268144</v>
-      </c>
-      <c r="R10">
-        <v>3741856</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>GP01</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Meridian Growth GP III LLC</v>
-      </c>
-      <c r="C11">
-        <v>1000000</v>
-      </c>
-      <c r="D11">
-        <v>650000</v>
-      </c>
-      <c r="E11">
-        <v>350000</v>
-      </c>
-      <c r="F11">
-        <v>64583.33</v>
-      </c>
-      <c r="G11">
-        <v>35416.67</v>
-      </c>
-      <c r="H11">
-        <v>13020.83</v>
-      </c>
-      <c r="I11">
-        <v>2968.75</v>
-      </c>
-      <c r="J11">
-        <v>1250</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>0</v>
-      </c>
-      <c r="O11">
-        <v>117239.58</v>
-      </c>
-      <c r="P11">
-        <v>115989.58</v>
-      </c>
-      <c r="Q11">
-        <v>534010.42</v>
-      </c>
-      <c r="R11">
-        <v>467239.58</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v>TOTAL</v>
-      </c>
-      <c r="C12">
-        <v>96000000</v>
-      </c>
-      <c r="D12">
-        <v>62400000</v>
-      </c>
-      <c r="E12">
-        <v>33600000</v>
-      </c>
-      <c r="F12">
-        <v>6200000</v>
-      </c>
-      <c r="G12">
-        <v>3400000</v>
-      </c>
-      <c r="H12">
-        <v>1250000</v>
-      </c>
-      <c r="I12">
-        <v>285000</v>
-      </c>
-      <c r="J12">
-        <v>120000</v>
-      </c>
-      <c r="K12" t="str">
-        <v/>
-      </c>
-      <c r="L12">
-        <v>126857.5</v>
-      </c>
-      <c r="M12">
-        <v>80500</v>
-      </c>
-      <c r="N12">
-        <v>46357.5</v>
-      </c>
-      <c r="O12">
-        <v>11301357.5</v>
-      </c>
-      <c r="P12">
-        <v>11181357.5</v>
-      </c>
-      <c r="Q12">
-        <v>51218642.5</v>
-      </c>
-      <c r="R12">
-        <v>44901357.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R12"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(notices): drop the sentence about wiring instructions that do not exist
The fund's template directed the investor to remit "in accordance with the
wiring instructions provided with this notice". No wiring instructions are
provided with the notice, so that sentence was false — and false in the one
paragraph that asks somebody to move money, which is exactly where a limited
partner's fraud radar sits.

Removed rather than softened. The notice now states an amount and a date and
says nothing about how to pay, which is honest but still not actionable: an
investor cannot wire against it alone. Closing that gap needs the bank details
themselves, and the comment in notice.ts says to put the sentence back when
they exist and can actually accompany the notice. A test fails if it returns
before then.

Also regenerates the Meridian sample, whose signatory the user changed.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/meridian-growth-partners-iii-call-4.xlsx
+++ b/samples/meridian-growth-partners-iii-call-4.xlsx
@@ -660,7 +660,7 @@
         <v>Signatory_Name</v>
       </c>
       <c r="B16" t="str">
-        <v>Priya Raghunathan</v>
+        <v>Baljeet Singh</v>
       </c>
       <c r="C16" t="str">
         <v>Who signs the notice.</v>
@@ -671,7 +671,7 @@
         <v>Signatory_Title</v>
       </c>
       <c r="B17" t="str">
-        <v>Chief Financial Officer</v>
+        <v>Fund Manager</v>
       </c>
       <c r="C17" t="str">
         <v>Their title, under the name.</v>

</xml_diff>